<commit_message>
#4912 Batch job mechanism - changed excel template + removed code for reports auto generation
</commit_message>
<xml_diff>
--- a/wp-content/themes/bp-child/groups/templates/SuperStreamTestProgress.xlsx
+++ b/wp-content/themes/bp-child/groups/templates/SuperStreamTestProgress.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Employer" sheetId="1" state="visible" r:id="rId2"/>
@@ -17,12 +17,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="20">
   <si>
     <t>Test Tracking Report For:</t>
   </si>
   <si>
     <t>SuperStream Community</t>
+  </si>
+  <si>
+    <t>Generated:</t>
   </si>
   <si>
     <t>Company</t>
@@ -349,7 +352,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col collapsed="false" hidden="false" max="1" min="1" style="0" width="29.837037037037"/>
@@ -393,93 +396,115 @@
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
     </row>
-    <row r="2" s="7" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+    <row r="2" s="3" customFormat="true" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="5" t="s">
+      <c r="B2" s="1"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+    </row>
+    <row r="3" s="7" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="6" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="5" t="s">
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="4" t="s">
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" s="12" customFormat="true" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
+      <c r="P3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="8" t="s">
+    </row>
+    <row r="4" s="12" customFormat="true" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="B4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="10" t="s">
+      <c r="C4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="D4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="F4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="G4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="H4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="I4" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="J4" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="10" t="s">
+      <c r="K4" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="M3" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="N3" s="9" t="s">
+      <c r="L4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="M4" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="P3" s="5"/>
+      <c r="N4" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="P4" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:P1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="G2:J2"/>
-    <mergeCell ref="K2:N2"/>
-    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="C2:P2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="K3:N3"/>
+    <mergeCell ref="P3:P4"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -496,7 +521,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col collapsed="false" hidden="false" max="1" min="1" style="0" width="29.837037037037"/>
@@ -540,93 +565,115 @@
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
     </row>
-    <row r="2" s="7" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+    <row r="2" s="3" customFormat="true" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="5" t="s">
+      <c r="B2" s="1"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+    </row>
+    <row r="3" s="7" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="6" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="5" t="s">
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="4" t="s">
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" s="12" customFormat="true" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
+      <c r="P3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="8" t="s">
+    </row>
+    <row r="4" s="12" customFormat="true" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="B4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="10" t="s">
+      <c r="C4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="D4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="F4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="G4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="H4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="I4" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="J4" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="10" t="s">
+      <c r="K4" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="M3" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="N3" s="9" t="s">
+      <c r="L4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="M4" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="P3" s="5"/>
+      <c r="N4" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="P4" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:P1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="G2:J2"/>
-    <mergeCell ref="K2:N2"/>
-    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="C2:P2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="K3:N3"/>
+    <mergeCell ref="P3:P4"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -643,7 +690,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col collapsed="false" hidden="false" max="1" min="1" style="0" width="29.837037037037"/>
@@ -687,93 +734,115 @@
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
     </row>
-    <row r="2" s="7" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+    <row r="2" s="3" customFormat="true" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="5" t="s">
+      <c r="B2" s="1"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+    </row>
+    <row r="3" s="7" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="6" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="5" t="s">
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="4" t="s">
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" s="12" customFormat="true" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
+      <c r="P3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="8" t="s">
+    </row>
+    <row r="4" s="12" customFormat="true" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="B4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="10" t="s">
+      <c r="C4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="D4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="F4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="G4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="H4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="I4" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="J4" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="10" t="s">
+      <c r="K4" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="M3" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="N3" s="9" t="s">
+      <c r="L4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="M4" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="P3" s="5"/>
+      <c r="N4" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="P4" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:P1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="G2:J2"/>
-    <mergeCell ref="K2:N2"/>
-    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="C2:P2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="K3:N3"/>
+    <mergeCell ref="P3:P4"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>